<commit_message>
users can support multiple days
</commit_message>
<xml_diff>
--- a/schedule/static/RgendaUsers.xlsx
+++ b/schedule/static/RgendaUsers.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="26311"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Allison.chen\Desktop\報帳\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/max.chen/PycharmProjects/skuld/schedule/static/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8355"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="16120"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,17 @@
     <definedName name="性別">#REF!</definedName>
     <definedName name="性別設定">list!$A$1:$A$2</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" concurrentCalc="0"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
+      <mx:ArchID Flags="2"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="61">
   <si>
     <t>電子信箱</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -224,6 +229,43 @@
   <si>
     <t>妊娠或哺乳期</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TEST001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>test001@gmail.com</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TEST001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>測試一</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>健檢診所</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>測試</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nn</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>男</t>
+  </si>
+  <si>
+    <t>使用者</t>
+  </si>
+  <si>
+    <t>正職人員</t>
   </si>
 </sst>
 </file>
@@ -300,16 +342,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -318,7 +360,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -333,6 +375,8 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -549,18 +593,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
+  <sheetPr enableFormatConditionsCalculation="0">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:O28"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="15" width="12.7109375" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="14.42578125" style="1"/>
+    <col min="1" max="1" width="5.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="15" width="12.6640625" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="14.5" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -654,7 +698,7 @@
         <v>40179</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="13.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
@@ -701,24 +745,52 @@
         <v>43831</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="13.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
+      <c r="B4" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="7">
+        <v>123456</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="O4" s="9">
+        <v>43831</v>
+      </c>
     </row>
     <row r="5" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1182,9 +1254,10 @@
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1"/>
     <hyperlink ref="D2" r:id="rId2"/>
+    <hyperlink ref="D4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
@@ -1227,20 +1300,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A1" s="6"/>
     </row>
-    <row r="2" spans="1:6" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A2" s="6"/>
     </row>
-    <row r="8" spans="1:6" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.15">
       <c r="B8" s="6" t="s">
         <v>40</v>
       </c>
@@ -1257,7 +1330,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.15">
       <c r="B9" s="6" t="s">
         <v>41</v>
       </c>
@@ -1274,22 +1347,22 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
       <c r="D10" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
       <c r="D11" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
       <c r="D12" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
       <c r="D13" s="6" t="s">
         <v>31</v>
       </c>

</xml_diff>